<commit_message>
v0.5.5: Feed LTM revenue & Adj. EBITDA into cap table D47/D48
Run ltm-metrics before captable so its LTM revenue and Adj. EBITDA
bridge totals flow into the cap table's LTM valuation column. captable
writes them to D47/D48 as =<value>*F7 (FX-converted to the F5 output
currency, in millions), falling back to the CapIQ IQ_REV/SP_EBITDA
formulas when no LTM values are supplied (standalone /captable or a plan
with no ltm-metrics stage). Swaps in the revised cap-table template
(D47/D48 empty, __snloffice helper tab re-stripped) and widens the
overview-slide picture range B15:F36 -> B15:F40 to include the Valuation
Metrics rows.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-beta/templates/INFOR Cap Table Template.xlsx
+++ b/infor-beta/templates/INFOR Cap Table Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="57255" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28455" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cap with Links" sheetId="1" state="visible" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Cap with Links'!$A$1:$T$187</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" calcMode="manual" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -72,7 +72,7 @@
     <numFmt numFmtId="182" formatCode="&quot;$&quot;#,##0.0_);\(&quot;$&quot;#,##0.0\);\-\-_);&quot;--&quot;_)"/>
     <numFmt numFmtId="183" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\);&quot;--&quot;"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -252,12 +252,6 @@
       <charset val="1"/>
       <b val="1"/>
       <color indexed="81"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Palatino Linotype"/>
-      <family val="1"/>
-      <color indexed="20"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -542,7 +536,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="7"/>
   </cellStyleXfs>
-  <cellXfs count="186">
+  <cellXfs count="184">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -877,9 +871,6 @@
     <xf numFmtId="165" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="176" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -958,8 +949,8 @@
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" vertical="center" indent="1"/>
@@ -968,9 +959,6 @@
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="171" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
@@ -1385,7 +1373,7 @@
         </is>
       </c>
       <c r="B1" s="63" t="n"/>
-      <c r="C1" s="133" t="n"/>
+      <c r="C1" s="132" t="n"/>
       <c r="G1" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -1475,14 +1463,14 @@
       <c r="C7" s="87" t="n"/>
       <c r="D7" s="87" t="n"/>
       <c r="E7" s="87" t="n"/>
-      <c r="F7" s="134" t="n"/>
+      <c r="F7" s="133" t="n"/>
       <c r="H7" s="66" t="n"/>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="8" t="n"/>
     </row>
     <row r="8" ht="3" customFormat="1" customHeight="1" s="4">
       <c r="B8" s="97" t="n"/>
-      <c r="F8" s="135" t="n"/>
+      <c r="F8" s="134" t="n"/>
       <c r="H8" s="66" t="n"/>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="8" t="n"/>
@@ -1496,7 +1484,7 @@
       <c r="C9" s="103" t="n"/>
       <c r="D9" s="103" t="n"/>
       <c r="E9" s="103" t="n"/>
-      <c r="F9" s="135" t="n"/>
+      <c r="F9" s="134" t="n"/>
       <c r="H9" s="66" t="n"/>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="8" t="n"/>
@@ -1536,7 +1524,7 @@
     </row>
     <row r="12" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="B12" s="87" t="n"/>
-      <c r="F12" s="136" t="n"/>
+      <c r="F12" s="135" t="n"/>
       <c r="H12" s="66" t="n"/>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="8" t="n"/>
@@ -1577,7 +1565,7 @@
         <f>CONCATENATE("Share Price (",TEXT(F6,"dd-mmm-yy"),")")</f>
         <v/>
       </c>
-      <c r="F16" s="137" t="n"/>
+      <c r="F16" s="136" t="n"/>
       <c r="H16" s="66" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -1586,7 +1574,7 @@
           <t>Basic Shares Outstanding</t>
         </is>
       </c>
-      <c r="F17" s="138">
+      <c r="F17" s="137">
         <f>F186</f>
         <v/>
       </c>
@@ -1600,7 +1588,7 @@
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
       <c r="E18" s="14" t="n"/>
-      <c r="F18" s="139">
+      <c r="F18" s="138">
         <f>F16*F17</f>
         <v/>
       </c>
@@ -1619,7 +1607,7 @@
         <f>IF(F10="Treasury Stock","Net","")&amp;" ITM Dilutive Securities"</f>
         <v/>
       </c>
-      <c r="F19" s="138">
+      <c r="F19" s="137">
         <f>IF(F10="Treasury Stock",F86,F84)</f>
         <v/>
       </c>
@@ -1630,7 +1618,7 @@
           <t>ITM Convertible Debentures</t>
         </is>
       </c>
-      <c r="F20" s="138">
+      <c r="F20" s="137">
         <f>F104</f>
         <v/>
       </c>
@@ -1644,7 +1632,7 @@
       <c r="C21" s="14" t="n"/>
       <c r="D21" s="14" t="n"/>
       <c r="E21" s="14" t="n"/>
-      <c r="F21" s="140">
+      <c r="F21" s="139">
         <f>F17+F19+F20</f>
         <v/>
       </c>
@@ -1667,7 +1655,7 @@
       <c r="C22" s="16" t="n"/>
       <c r="D22" s="16" t="n"/>
       <c r="E22" s="16" t="n"/>
-      <c r="F22" s="141">
+      <c r="F22" s="140">
         <f>F16*F21</f>
         <v/>
       </c>
@@ -1701,7 +1689,7 @@
           <t>Add: Debt</t>
         </is>
       </c>
-      <c r="F24" s="142">
+      <c r="F24" s="141">
         <f>F122*F7</f>
         <v/>
       </c>
@@ -1721,7 +1709,7 @@
           <t>Add: Leases</t>
         </is>
       </c>
-      <c r="F25" s="142">
+      <c r="F25" s="141">
         <f>IF($F$11="ON",$F$143,0)*F7</f>
         <v/>
       </c>
@@ -1741,7 +1729,7 @@
           <t>Less: Cash</t>
         </is>
       </c>
-      <c r="F26" s="142">
+      <c r="F26" s="141">
         <f>-F164*F7</f>
         <v/>
       </c>
@@ -1761,7 +1749,7 @@
           <t>Less: Cash from ITM Proceeds</t>
         </is>
       </c>
-      <c r="F27" s="142">
+      <c r="F27" s="141">
         <f>IF(F10="Treasury Stock",0,-F82)*F7</f>
         <v/>
       </c>
@@ -1784,7 +1772,7 @@
       <c r="C28" s="65" t="n"/>
       <c r="D28" s="65" t="n"/>
       <c r="E28" s="65" t="n"/>
-      <c r="F28" s="143">
+      <c r="F28" s="142">
         <f>F24+F25+F26+F27</f>
         <v/>
       </c>
@@ -1806,8 +1794,8 @@
       </c>
       <c r="C29" s="18" t="n"/>
       <c r="D29" s="18" t="n"/>
-      <c r="E29" s="144" t="n"/>
-      <c r="F29" s="145">
+      <c r="E29" s="143" t="n"/>
+      <c r="F29" s="144">
         <f>+$F$52*F7</f>
         <v/>
       </c>
@@ -1831,8 +1819,8 @@
       </c>
       <c r="C30" s="20" t="n"/>
       <c r="D30" s="20" t="n"/>
-      <c r="E30" s="146" t="n"/>
-      <c r="F30" s="145">
+      <c r="E30" s="145" t="n"/>
+      <c r="F30" s="144">
         <f>+$F$53*F7</f>
         <v/>
       </c>
@@ -1857,7 +1845,7 @@
       <c r="C31" s="16" t="n"/>
       <c r="D31" s="16" t="n"/>
       <c r="E31" s="16" t="n"/>
-      <c r="F31" s="141">
+      <c r="F31" s="140">
         <f>F22+F28+F29+F30</f>
         <v/>
       </c>
@@ -1874,9 +1862,9 @@
     <row r="32" ht="18" customHeight="1" thickTop="1">
       <c r="B32" s="94" t="n"/>
       <c r="C32" s="105" t="n"/>
-      <c r="D32" s="147" t="n"/>
-      <c r="E32" s="147" t="n"/>
-      <c r="F32" s="147" t="n"/>
+      <c r="D32" s="146" t="n"/>
+      <c r="E32" s="146" t="n"/>
+      <c r="F32" s="146" t="n"/>
     </row>
     <row r="33" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="B33" s="104" t="inlineStr">
@@ -1885,17 +1873,17 @@
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
-      <c r="D33" s="148" t="inlineStr">
+      <c r="D33" s="147" t="inlineStr">
         <is>
           <t>LTM</t>
         </is>
       </c>
-      <c r="E33" s="149" t="inlineStr">
+      <c r="E33" s="148" t="inlineStr">
         <is>
           <t>CY2026</t>
         </is>
       </c>
-      <c r="F33" s="149" t="inlineStr">
+      <c r="F33" s="148" t="inlineStr">
         <is>
           <t>CY2027</t>
         </is>
@@ -1909,15 +1897,15 @@
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
-      <c r="D34" s="150">
+      <c r="D34" s="149">
         <f>IFERROR(IF(D47="NULL","na ",D47),"n/a ")</f>
         <v/>
       </c>
-      <c r="E34" s="142">
+      <c r="E34" s="141">
         <f>IFERROR(IF(E47="NULL","na ",E47),"n/a ")</f>
         <v/>
       </c>
-      <c r="F34" s="142">
+      <c r="F34" s="141">
         <f>IFERROR(IF(F47="NULL","na ",F47),"n/a ")</f>
         <v/>
       </c>
@@ -1930,15 +1918,15 @@
         </is>
       </c>
       <c r="C35" s="10" t="n"/>
-      <c r="D35" s="150">
+      <c r="D35" s="149">
         <f>IFERROR(IF(D48="NULL","na ",D48),"na/ ")</f>
         <v/>
       </c>
-      <c r="E35" s="142">
+      <c r="E35" s="141">
         <f>IFERROR(IF(E48="NULL","na ",E48),"na/ ")</f>
         <v/>
       </c>
-      <c r="F35" s="142">
+      <c r="F35" s="141">
         <f>IFERROR(IF(F48="NULL","na ",F48),"na/ ")</f>
         <v/>
       </c>
@@ -1951,15 +1939,15 @@
         </is>
       </c>
       <c r="C36" s="10" t="n"/>
-      <c r="D36" s="151">
+      <c r="D36" s="150">
         <f>IFERROR(IF(D35&lt;0,"nmf ",D35/D34),"n/a ")</f>
         <v/>
       </c>
-      <c r="E36" s="151">
+      <c r="E36" s="150">
         <f>IFERROR(IF(E35&lt;0,"nmf ",E35/E34),"n/a ")</f>
         <v/>
       </c>
-      <c r="F36" s="151">
+      <c r="F36" s="150">
         <f>IFERROR(IF(F35&lt;0,"nmf ",F35/F34),"n/a ")</f>
         <v/>
       </c>
@@ -1968,9 +1956,9 @@
     <row r="37" ht="3" customFormat="1" customHeight="1" s="4">
       <c r="B37" s="111" t="n"/>
       <c r="C37" s="10" t="n"/>
-      <c r="D37" s="152" t="n"/>
-      <c r="E37" s="152" t="n"/>
-      <c r="F37" s="152" t="n"/>
+      <c r="D37" s="151" t="n"/>
+      <c r="E37" s="151" t="n"/>
+      <c r="F37" s="151" t="n"/>
       <c r="H37" s="66" t="n"/>
     </row>
     <row r="38" ht="18" customFormat="1" customHeight="1" s="4">
@@ -1988,15 +1976,15 @@
           <t>EV / Revenue</t>
         </is>
       </c>
-      <c r="D39" s="153">
+      <c r="D39" s="152">
         <f>+$F$31/D$34</f>
         <v/>
       </c>
-      <c r="E39" s="153">
+      <c r="E39" s="152">
         <f>+$F$31/E$34</f>
         <v/>
       </c>
-      <c r="F39" s="153">
+      <c r="F39" s="152">
         <f>+$F$31/F$34</f>
         <v/>
       </c>
@@ -2008,15 +1996,15 @@
           <t>EV / Adj. EBITDA</t>
         </is>
       </c>
-      <c r="D40" s="153">
+      <c r="D40" s="152">
         <f>+$F$31/D$35</f>
         <v/>
       </c>
-      <c r="E40" s="153">
+      <c r="E40" s="152">
         <f>+$F$31/E$35</f>
         <v/>
       </c>
-      <c r="F40" s="153">
+      <c r="F40" s="152">
         <f>+$F$31/F$35</f>
         <v/>
       </c>
@@ -2024,9 +2012,9 @@
     </row>
     <row r="41" ht="3" customFormat="1" customHeight="1" s="4">
       <c r="B41" s="111" t="n"/>
-      <c r="D41" s="154" t="n"/>
-      <c r="E41" s="154" t="n"/>
-      <c r="F41" s="154" t="n"/>
+      <c r="D41" s="153" t="n"/>
+      <c r="E41" s="153" t="n"/>
+      <c r="F41" s="153" t="n"/>
       <c r="H41" s="66" t="n"/>
     </row>
     <row r="42" ht="18" customFormat="1" customHeight="1" s="4">
@@ -2035,9 +2023,9 @@
           <t>Street Metrics</t>
         </is>
       </c>
-      <c r="D42" s="154" t="n"/>
-      <c r="E42" s="154" t="n"/>
-      <c r="F42" s="154" t="n"/>
+      <c r="D42" s="153" t="n"/>
+      <c r="E42" s="153" t="n"/>
+      <c r="F42" s="153" t="n"/>
       <c r="H42" s="66" t="n"/>
     </row>
     <row r="43" ht="18" customFormat="1" customHeight="1" s="4">
@@ -2046,9 +2034,9 @@
           <t>Analyst Coverage (# of Analysts)</t>
         </is>
       </c>
-      <c r="D43" s="154" t="n"/>
-      <c r="E43" s="154" t="n"/>
-      <c r="F43" s="155">
+      <c r="D43" s="153" t="n"/>
+      <c r="E43" s="153" t="n"/>
+      <c r="F43" s="154">
         <f t="array" ref="F43">_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_NUM_BROKER_REC",$F$6,"Options:NA=NA")</f>
         <v/>
       </c>
@@ -2065,9 +2053,9 @@
           <t>Average Target Price</t>
         </is>
       </c>
-      <c r="D44" s="154" t="n"/>
-      <c r="E44" s="154" t="n"/>
-      <c r="F44" s="156">
+      <c r="D44" s="153" t="n"/>
+      <c r="E44" s="153" t="n"/>
+      <c r="F44" s="155">
         <f t="array" ref="F44">_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_PRICE_TARGET",$F$6,"Options: NA=NA,Curr="&amp;$F$4)</f>
         <v/>
       </c>
@@ -2079,9 +2067,9 @@
           <t>% Upside vs. Current</t>
         </is>
       </c>
-      <c r="D45" s="154" t="n"/>
-      <c r="E45" s="154" t="n"/>
-      <c r="F45" s="157">
+      <c r="D45" s="153" t="n"/>
+      <c r="E45" s="153" t="n"/>
+      <c r="F45" s="156">
         <f>IFERROR(F44/F16-1,"na ")</f>
         <v/>
       </c>
@@ -2090,9 +2078,9 @@
     <row r="46" ht="18" customFormat="1" customHeight="1" s="4">
       <c r="B46" s="111" t="n"/>
       <c r="C46" s="10" t="n"/>
-      <c r="D46" s="158" t="n"/>
-      <c r="E46" s="158" t="n"/>
-      <c r="F46" s="158" t="n"/>
+      <c r="D46" s="157" t="n"/>
+      <c r="E46" s="157" t="n"/>
+      <c r="F46" s="157" t="n"/>
       <c r="H46" s="66" t="n"/>
     </row>
     <row r="47" ht="18" customFormat="1" customHeight="1" s="4">
@@ -2102,15 +2090,12 @@
         </is>
       </c>
       <c r="C47" s="10" t="n"/>
-      <c r="D47" s="159">
-        <f>_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"IQ_REV",D$33,$F$6,"Options:Mag=Millions,NA=NA,Curr="&amp;$F$5)</f>
-        <v/>
-      </c>
-      <c r="E47" s="160">
+      <c r="D47" s="158" t="n"/>
+      <c r="E47" s="159">
         <f t="array" ref="E47">_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_REV_EST",E$33,$F$6,"Options:Mag=Millions,NA=NA,Curr="&amp;$F$5)</f>
         <v/>
       </c>
-      <c r="F47" s="160">
+      <c r="F47" s="159">
         <f t="array" ref="F47">_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_REV_EST",F$33,$F$6,"Options:Mag=Millions,NA=NA,Curr="&amp;$F$5)</f>
         <v/>
       </c>
@@ -2123,15 +2108,12 @@
         </is>
       </c>
       <c r="C48" s="10" t="n"/>
-      <c r="D48" s="159">
-        <f>_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_EBITDA",D$33,$F$6,"Options:Mag=Millions,NA=NA,Curr="&amp;$F$5)</f>
-        <v/>
-      </c>
-      <c r="E48" s="160">
+      <c r="D48" s="158" t="n"/>
+      <c r="E48" s="159">
         <f t="array" ref="E48">_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_EBITDA_EST",E$33,$F$6,"Options:Mag=Millions,NA=NA,Curr="&amp;$F$5)</f>
         <v/>
       </c>
-      <c r="F48" s="160">
+      <c r="F48" s="159">
         <f t="array" ref="F48">_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_EBITDA_EST",F$33,$F$6,"Options:Mag=Millions,NA=NA,Curr="&amp;$F$5)</f>
         <v/>
       </c>
@@ -2140,9 +2122,9 @@
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="12" t="n"/>
       <c r="C49" s="10" t="n"/>
-      <c r="D49" s="161" t="n"/>
-      <c r="E49" s="161" t="n"/>
-      <c r="F49" s="161" t="n"/>
+      <c r="D49" s="160" t="n"/>
+      <c r="E49" s="160" t="n"/>
+      <c r="F49" s="160" t="n"/>
       <c r="Q49" s="4" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -2184,8 +2166,8 @@
         </is>
       </c>
       <c r="D52" s="13" t="n"/>
-      <c r="E52" s="162" t="n"/>
-      <c r="F52" s="163" t="n"/>
+      <c r="E52" s="161" t="n"/>
+      <c r="F52" s="158" t="n"/>
       <c r="Q52" s="4" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1">
@@ -2195,15 +2177,15 @@
         </is>
       </c>
       <c r="D53" s="13" t="n"/>
-      <c r="E53" s="162" t="n"/>
-      <c r="F53" s="163" t="n"/>
+      <c r="E53" s="161" t="n"/>
+      <c r="F53" s="158" t="n"/>
       <c r="Q53" s="4" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="B54" s="12" t="n"/>
       <c r="D54" s="13" t="n"/>
       <c r="E54" s="13" t="n"/>
-      <c r="F54" s="154" t="n"/>
+      <c r="F54" s="153" t="n"/>
       <c r="Q54" s="4" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" thickBot="1">
@@ -2248,13 +2230,13 @@
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="B57" s="24" t="n"/>
-      <c r="C57" s="164" t="n"/>
+      <c r="C57" s="162" t="n"/>
       <c r="D57" s="26" t="n"/>
-      <c r="E57" s="165">
+      <c r="E57" s="163">
         <f>IF(D57&lt;F$16,C57,0)</f>
         <v/>
       </c>
-      <c r="F57" s="166">
+      <c r="F57" s="164">
         <f>E57*D57</f>
         <v/>
       </c>
@@ -2262,13 +2244,13 @@
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="B58" s="24" t="n"/>
-      <c r="C58" s="164" t="n"/>
+      <c r="C58" s="162" t="n"/>
       <c r="D58" s="26" t="n"/>
-      <c r="E58" s="165">
+      <c r="E58" s="163">
         <f>IF(D58&lt;F$16,C58,0)</f>
         <v/>
       </c>
-      <c r="F58" s="166">
+      <c r="F58" s="164">
         <f>E58*D58</f>
         <v/>
       </c>
@@ -2277,13 +2259,13 @@
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="B59" s="24" t="n"/>
-      <c r="C59" s="164" t="n"/>
+      <c r="C59" s="162" t="n"/>
       <c r="D59" s="26" t="n"/>
-      <c r="E59" s="165">
+      <c r="E59" s="163">
         <f>IF(D59&lt;F$16,C59,0)</f>
         <v/>
       </c>
-      <c r="F59" s="166">
+      <c r="F59" s="164">
         <f>E59*D59</f>
         <v/>
       </c>
@@ -2292,13 +2274,13 @@
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="B60" s="24" t="n"/>
-      <c r="C60" s="164" t="n"/>
+      <c r="C60" s="162" t="n"/>
       <c r="D60" s="26" t="n"/>
-      <c r="E60" s="165">
+      <c r="E60" s="163">
         <f>IF(D60&lt;F$16,C60,0)</f>
         <v/>
       </c>
-      <c r="F60" s="166">
+      <c r="F60" s="164">
         <f>E60*D60</f>
         <v/>
       </c>
@@ -2306,13 +2288,13 @@
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="B61" s="24" t="n"/>
-      <c r="C61" s="164" t="n"/>
+      <c r="C61" s="162" t="n"/>
       <c r="D61" s="26" t="n"/>
-      <c r="E61" s="165">
+      <c r="E61" s="163">
         <f>IF(D61&lt;F$16,C61,0)</f>
         <v/>
       </c>
-      <c r="F61" s="166">
+      <c r="F61" s="164">
         <f>E61*D61</f>
         <v/>
       </c>
@@ -2320,13 +2302,13 @@
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="B62" s="24" t="n"/>
-      <c r="C62" s="164" t="n"/>
+      <c r="C62" s="162" t="n"/>
       <c r="D62" s="26" t="n"/>
-      <c r="E62" s="165">
+      <c r="E62" s="163">
         <f>IF(D62&lt;F$16,C62,0)</f>
         <v/>
       </c>
-      <c r="F62" s="166">
+      <c r="F62" s="164">
         <f>E62*D62</f>
         <v/>
       </c>
@@ -2334,13 +2316,13 @@
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="B63" s="24" t="n"/>
-      <c r="C63" s="164" t="n"/>
+      <c r="C63" s="162" t="n"/>
       <c r="D63" s="26" t="n"/>
-      <c r="E63" s="165">
+      <c r="E63" s="163">
         <f>IF(D63&lt;F$16,C63,0)</f>
         <v/>
       </c>
-      <c r="F63" s="166">
+      <c r="F63" s="164">
         <f>E63*D63</f>
         <v/>
       </c>
@@ -2348,13 +2330,13 @@
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="B64" s="24" t="n"/>
-      <c r="C64" s="164" t="n"/>
+      <c r="C64" s="162" t="n"/>
       <c r="D64" s="26" t="n"/>
-      <c r="E64" s="165">
+      <c r="E64" s="163">
         <f>IF(D64&lt;F$16,C64,0)</f>
         <v/>
       </c>
-      <c r="F64" s="166">
+      <c r="F64" s="164">
         <f>E64*D64</f>
         <v/>
       </c>
@@ -2362,13 +2344,13 @@
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="B65" s="24" t="n"/>
-      <c r="C65" s="164" t="n"/>
+      <c r="C65" s="162" t="n"/>
       <c r="D65" s="26" t="n"/>
-      <c r="E65" s="165">
+      <c r="E65" s="163">
         <f>IF(D65&lt;F$16,C65,0)</f>
         <v/>
       </c>
-      <c r="F65" s="166">
+      <c r="F65" s="164">
         <f>E65*D65</f>
         <v/>
       </c>
@@ -2376,13 +2358,13 @@
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="B66" s="24" t="n"/>
-      <c r="C66" s="164" t="n"/>
+      <c r="C66" s="162" t="n"/>
       <c r="D66" s="26" t="n"/>
-      <c r="E66" s="165">
+      <c r="E66" s="163">
         <f>IF(D66&lt;F$16,C66,0)</f>
         <v/>
       </c>
-      <c r="F66" s="166">
+      <c r="F66" s="164">
         <f>E66*D66</f>
         <v/>
       </c>
@@ -2390,13 +2372,13 @@
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="B67" s="24" t="n"/>
-      <c r="C67" s="164" t="n"/>
+      <c r="C67" s="162" t="n"/>
       <c r="D67" s="26" t="n"/>
-      <c r="E67" s="165">
+      <c r="E67" s="163">
         <f>IF(D67&lt;F$16,C67,0)</f>
         <v/>
       </c>
-      <c r="F67" s="166">
+      <c r="F67" s="164">
         <f>E67*D67</f>
         <v/>
       </c>
@@ -2404,13 +2386,13 @@
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="B68" s="24" t="n"/>
-      <c r="C68" s="164" t="n"/>
+      <c r="C68" s="162" t="n"/>
       <c r="D68" s="26" t="n"/>
-      <c r="E68" s="165">
+      <c r="E68" s="163">
         <f>IF(D68&lt;F$16,C68,0)</f>
         <v/>
       </c>
-      <c r="F68" s="166">
+      <c r="F68" s="164">
         <f>E68*D68</f>
         <v/>
       </c>
@@ -2418,13 +2400,13 @@
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="B69" s="24" t="n"/>
-      <c r="C69" s="164" t="n"/>
+      <c r="C69" s="162" t="n"/>
       <c r="D69" s="26" t="n"/>
-      <c r="E69" s="165">
+      <c r="E69" s="163">
         <f>IF(D69&lt;F$16,C69,0)</f>
         <v/>
       </c>
-      <c r="F69" s="166">
+      <c r="F69" s="164">
         <f>E69*D69</f>
         <v/>
       </c>
@@ -2432,13 +2414,13 @@
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="B70" s="24" t="n"/>
-      <c r="C70" s="164" t="n"/>
+      <c r="C70" s="162" t="n"/>
       <c r="D70" s="26" t="n"/>
-      <c r="E70" s="165">
+      <c r="E70" s="163">
         <f>IF(D70&lt;F$16,C70,0)</f>
         <v/>
       </c>
-      <c r="F70" s="166">
+      <c r="F70" s="164">
         <f>E70*D70</f>
         <v/>
       </c>
@@ -2446,13 +2428,13 @@
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="B71" s="24" t="n"/>
-      <c r="C71" s="164" t="n"/>
+      <c r="C71" s="162" t="n"/>
       <c r="D71" s="26" t="n"/>
-      <c r="E71" s="165">
+      <c r="E71" s="163">
         <f>IF(D71&lt;F$16,C71,0)</f>
         <v/>
       </c>
-      <c r="F71" s="166">
+      <c r="F71" s="164">
         <f>E71*D71</f>
         <v/>
       </c>
@@ -2460,13 +2442,13 @@
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="B72" s="24" t="n"/>
-      <c r="C72" s="164" t="n"/>
+      <c r="C72" s="162" t="n"/>
       <c r="D72" s="26" t="n"/>
-      <c r="E72" s="165">
+      <c r="E72" s="163">
         <f>IF(D72&lt;F$16,C72,0)</f>
         <v/>
       </c>
-      <c r="F72" s="166">
+      <c r="F72" s="164">
         <f>E72*D72</f>
         <v/>
       </c>
@@ -2474,13 +2456,13 @@
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="B73" s="24" t="n"/>
-      <c r="C73" s="164" t="n"/>
+      <c r="C73" s="162" t="n"/>
       <c r="D73" s="26" t="n"/>
-      <c r="E73" s="165">
+      <c r="E73" s="163">
         <f>IF(D73&lt;F$16,C73,0)</f>
         <v/>
       </c>
-      <c r="F73" s="166">
+      <c r="F73" s="164">
         <f>E73*D73</f>
         <v/>
       </c>
@@ -2488,13 +2470,13 @@
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="B74" s="24" t="n"/>
-      <c r="C74" s="164" t="n"/>
+      <c r="C74" s="162" t="n"/>
       <c r="D74" s="26" t="n"/>
-      <c r="E74" s="165">
+      <c r="E74" s="163">
         <f>IF(D74&lt;F$16,C74,0)</f>
         <v/>
       </c>
-      <c r="F74" s="166">
+      <c r="F74" s="164">
         <f>E74*D74</f>
         <v/>
       </c>
@@ -2502,91 +2484,91 @@
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="B75" s="24" t="n"/>
-      <c r="C75" s="164" t="n"/>
+      <c r="C75" s="162" t="n"/>
       <c r="D75" s="26" t="n"/>
-      <c r="E75" s="165">
+      <c r="E75" s="163">
         <f>IF(D75&lt;F$16,C75,0)</f>
         <v/>
       </c>
-      <c r="F75" s="166">
+      <c r="F75" s="164">
         <f>E75*D75</f>
         <v/>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="B76" s="24" t="n"/>
-      <c r="C76" s="164" t="n"/>
+      <c r="C76" s="162" t="n"/>
       <c r="D76" s="26" t="n"/>
-      <c r="E76" s="165">
+      <c r="E76" s="163">
         <f>IF(D76&lt;F$16,C76,0)</f>
         <v/>
       </c>
-      <c r="F76" s="166">
+      <c r="F76" s="164">
         <f>E76*D76</f>
         <v/>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="B77" s="24" t="n"/>
-      <c r="C77" s="164" t="n"/>
+      <c r="C77" s="162" t="n"/>
       <c r="D77" s="26" t="n"/>
-      <c r="E77" s="165">
+      <c r="E77" s="163">
         <f>IF(D77&lt;F$16,C77,0)</f>
         <v/>
       </c>
-      <c r="F77" s="166">
+      <c r="F77" s="164">
         <f>E77*D77</f>
         <v/>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="B78" s="24" t="n"/>
-      <c r="C78" s="164" t="n"/>
+      <c r="C78" s="162" t="n"/>
       <c r="D78" s="26" t="n"/>
-      <c r="E78" s="165">
+      <c r="E78" s="163">
         <f>IF(D78&lt;F$16,C78,0)</f>
         <v/>
       </c>
-      <c r="F78" s="166">
+      <c r="F78" s="164">
         <f>E78*D78</f>
         <v/>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="B79" s="24" t="n"/>
-      <c r="C79" s="164" t="n"/>
+      <c r="C79" s="162" t="n"/>
       <c r="D79" s="26" t="n"/>
-      <c r="E79" s="165">
+      <c r="E79" s="163">
         <f>IF(D79&lt;F$16,C79,0)</f>
         <v/>
       </c>
-      <c r="F79" s="166">
+      <c r="F79" s="164">
         <f>E79*D79</f>
         <v/>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="B80" s="24" t="n"/>
-      <c r="C80" s="164" t="n"/>
+      <c r="C80" s="162" t="n"/>
       <c r="D80" s="26" t="n"/>
-      <c r="E80" s="165">
+      <c r="E80" s="163">
         <f>IF(D80&lt;F$16,C80,0)</f>
         <v/>
       </c>
-      <c r="F80" s="166">
+      <c r="F80" s="164">
         <f>E80*D80</f>
         <v/>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="B81" s="24" t="n"/>
-      <c r="C81" s="164" t="n"/>
+      <c r="C81" s="162" t="n"/>
       <c r="D81" s="26" t="n"/>
-      <c r="E81" s="165">
+      <c r="E81" s="163">
         <f>IF(D81&lt;F$16,C81,0)</f>
         <v/>
       </c>
-      <c r="F81" s="166">
+      <c r="F81" s="164">
         <f>E81*D81</f>
         <v/>
       </c>
@@ -2599,11 +2581,11 @@
       </c>
       <c r="C82" s="27" t="n"/>
       <c r="D82" s="27" t="n"/>
-      <c r="E82" s="167">
+      <c r="E82" s="165">
         <f>SUM(E57:E81)</f>
         <v/>
       </c>
-      <c r="F82" s="168">
+      <c r="F82" s="166">
         <f>SUM(F57:F81)</f>
         <v/>
       </c>
@@ -2616,7 +2598,7 @@
           <t>Total ITM Options, Warrants, etc.</t>
         </is>
       </c>
-      <c r="F84" s="165">
+      <c r="F84" s="163">
         <f>E82</f>
         <v/>
       </c>
@@ -2630,7 +2612,7 @@
       <c r="C85" s="17" t="n"/>
       <c r="D85" s="17" t="n"/>
       <c r="E85" s="17" t="n"/>
-      <c r="F85" s="169">
+      <c r="F85" s="167">
         <f>-F82/F16</f>
         <v/>
       </c>
@@ -2644,7 +2626,7 @@
       <c r="C86" s="27" t="n"/>
       <c r="D86" s="27" t="n"/>
       <c r="E86" s="27" t="n"/>
-      <c r="F86" s="167">
+      <c r="F86" s="165">
         <f>SUM(F84:F85)</f>
         <v/>
       </c>
@@ -2691,140 +2673,140 @@
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="B90" s="24" t="n"/>
-      <c r="C90" s="163" t="n"/>
-      <c r="D90" s="170" t="n"/>
-      <c r="E90" s="171" t="n"/>
-      <c r="F90" s="165">
+      <c r="C90" s="158" t="n"/>
+      <c r="D90" s="168" t="n"/>
+      <c r="E90" s="169" t="n"/>
+      <c r="F90" s="163">
         <f>IF(E90&lt;F$16,(C90/1000)*D90,0)</f>
         <v/>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="B91" s="24" t="n"/>
-      <c r="C91" s="163" t="n"/>
-      <c r="D91" s="172" t="n"/>
-      <c r="E91" s="171" t="n"/>
-      <c r="F91" s="165">
+      <c r="C91" s="158" t="n"/>
+      <c r="D91" s="170" t="n"/>
+      <c r="E91" s="169" t="n"/>
+      <c r="F91" s="163">
         <f>IF(E91&lt;F$16,(C91/1000)*D91,0)</f>
         <v/>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="B92" s="24" t="n"/>
-      <c r="C92" s="163" t="n"/>
-      <c r="D92" s="172" t="n"/>
-      <c r="E92" s="171" t="n"/>
-      <c r="F92" s="165">
+      <c r="C92" s="158" t="n"/>
+      <c r="D92" s="170" t="n"/>
+      <c r="E92" s="169" t="n"/>
+      <c r="F92" s="163">
         <f>IF(E92&lt;F$16,(C92/1000)*D92,0)</f>
         <v/>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="B93" s="24" t="n"/>
-      <c r="C93" s="163" t="n"/>
-      <c r="D93" s="172" t="n"/>
-      <c r="E93" s="171" t="n"/>
-      <c r="F93" s="165">
+      <c r="C93" s="158" t="n"/>
+      <c r="D93" s="170" t="n"/>
+      <c r="E93" s="169" t="n"/>
+      <c r="F93" s="163">
         <f>IF(E93&lt;F$16,(C93/1000)*D93,0)</f>
         <v/>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="B94" s="24" t="n"/>
-      <c r="C94" s="163" t="n"/>
-      <c r="D94" s="172" t="n"/>
-      <c r="E94" s="171" t="n"/>
-      <c r="F94" s="165">
+      <c r="C94" s="158" t="n"/>
+      <c r="D94" s="170" t="n"/>
+      <c r="E94" s="169" t="n"/>
+      <c r="F94" s="163">
         <f>IF(E94&lt;F$16,(C94/1000)*D94,0)</f>
         <v/>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="B95" s="24" t="n"/>
-      <c r="C95" s="163" t="n"/>
-      <c r="D95" s="172" t="n"/>
-      <c r="E95" s="171" t="n"/>
-      <c r="F95" s="165">
+      <c r="C95" s="158" t="n"/>
+      <c r="D95" s="170" t="n"/>
+      <c r="E95" s="169" t="n"/>
+      <c r="F95" s="163">
         <f>IF(E95&lt;F$16,(C95/1000)*D95,0)</f>
         <v/>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="B96" s="24" t="n"/>
-      <c r="C96" s="163" t="n"/>
-      <c r="D96" s="172" t="n"/>
-      <c r="E96" s="171" t="n"/>
-      <c r="F96" s="165">
+      <c r="C96" s="158" t="n"/>
+      <c r="D96" s="170" t="n"/>
+      <c r="E96" s="169" t="n"/>
+      <c r="F96" s="163">
         <f>IF(E96&lt;F$16,(C96/1000)*D96,0)</f>
         <v/>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="B97" s="24" t="n"/>
-      <c r="C97" s="163" t="n"/>
-      <c r="D97" s="172" t="n"/>
-      <c r="E97" s="171" t="n"/>
-      <c r="F97" s="165">
+      <c r="C97" s="158" t="n"/>
+      <c r="D97" s="170" t="n"/>
+      <c r="E97" s="169" t="n"/>
+      <c r="F97" s="163">
         <f>IF(E97&lt;F$16,(C97/1000)*D97,0)</f>
         <v/>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="B98" s="24" t="n"/>
-      <c r="C98" s="163" t="n"/>
-      <c r="D98" s="172" t="n"/>
-      <c r="E98" s="171" t="n"/>
-      <c r="F98" s="165">
+      <c r="C98" s="158" t="n"/>
+      <c r="D98" s="170" t="n"/>
+      <c r="E98" s="169" t="n"/>
+      <c r="F98" s="163">
         <f>IF(E98&lt;F$16,(C98/1000)*D98,0)</f>
         <v/>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="B99" s="24" t="n"/>
-      <c r="C99" s="163" t="n"/>
-      <c r="D99" s="172" t="n"/>
-      <c r="E99" s="171" t="n"/>
-      <c r="F99" s="165">
+      <c r="C99" s="158" t="n"/>
+      <c r="D99" s="170" t="n"/>
+      <c r="E99" s="169" t="n"/>
+      <c r="F99" s="163">
         <f>IF(E99&lt;F$16,(C99/1000)*D99,0)</f>
         <v/>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="B100" s="24" t="n"/>
-      <c r="C100" s="163" t="n"/>
-      <c r="D100" s="172" t="n"/>
-      <c r="E100" s="171" t="n"/>
-      <c r="F100" s="165">
+      <c r="C100" s="158" t="n"/>
+      <c r="D100" s="170" t="n"/>
+      <c r="E100" s="169" t="n"/>
+      <c r="F100" s="163">
         <f>IF(E100&lt;F$16,(C100/1000)*D100,0)</f>
         <v/>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="B101" s="24" t="n"/>
-      <c r="C101" s="163" t="n"/>
-      <c r="D101" s="172" t="n"/>
-      <c r="E101" s="171" t="n"/>
-      <c r="F101" s="165">
+      <c r="C101" s="158" t="n"/>
+      <c r="D101" s="170" t="n"/>
+      <c r="E101" s="169" t="n"/>
+      <c r="F101" s="163">
         <f>IF(E101&lt;F$16,(C101/1000)*D101,0)</f>
         <v/>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="B102" s="24" t="n"/>
-      <c r="C102" s="163" t="n"/>
-      <c r="D102" s="172" t="n"/>
-      <c r="E102" s="171" t="n"/>
-      <c r="F102" s="165">
+      <c r="C102" s="158" t="n"/>
+      <c r="D102" s="170" t="n"/>
+      <c r="E102" s="169" t="n"/>
+      <c r="F102" s="163">
         <f>IF(E102&lt;F$16,(C102/1000)*D102,0)</f>
         <v/>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="B103" s="24" t="n"/>
-      <c r="C103" s="163" t="n"/>
-      <c r="D103" s="172" t="n"/>
-      <c r="E103" s="171" t="n"/>
-      <c r="F103" s="165">
+      <c r="C103" s="158" t="n"/>
+      <c r="D103" s="170" t="n"/>
+      <c r="E103" s="169" t="n"/>
+      <c r="F103" s="163">
         <f>IF(E103&lt;F$16,(C103/1000)*D103,0)</f>
         <v/>
       </c>
@@ -2838,7 +2820,7 @@
       <c r="C104" s="27" t="n"/>
       <c r="D104" s="27" t="n"/>
       <c r="E104" s="27" t="n"/>
-      <c r="F104" s="167">
+      <c r="F104" s="165">
         <f>SUM(F90:F103)</f>
         <v/>
       </c>
@@ -2877,101 +2859,101 @@
     </row>
     <row r="108" ht="15" customHeight="1">
       <c r="B108" s="24" t="n"/>
-      <c r="C108" s="173" t="n"/>
-      <c r="D108" s="174" t="n"/>
-      <c r="E108" s="162" t="n"/>
-      <c r="F108" s="163" t="n"/>
+      <c r="C108" s="171" t="n"/>
+      <c r="D108" s="172" t="n"/>
+      <c r="E108" s="161" t="n"/>
+      <c r="F108" s="158" t="n"/>
     </row>
     <row r="109" ht="15" customHeight="1">
       <c r="B109" s="24" t="n"/>
-      <c r="C109" s="173" t="n"/>
-      <c r="D109" s="174" t="n"/>
-      <c r="E109" s="162" t="n"/>
-      <c r="F109" s="163" t="n"/>
+      <c r="C109" s="171" t="n"/>
+      <c r="D109" s="172" t="n"/>
+      <c r="E109" s="161" t="n"/>
+      <c r="F109" s="158" t="n"/>
     </row>
     <row r="110" ht="15" customHeight="1">
       <c r="B110" s="75" t="n"/>
-      <c r="C110" s="173" t="n"/>
-      <c r="D110" s="174" t="n"/>
-      <c r="E110" s="162" t="n"/>
-      <c r="F110" s="163" t="n"/>
+      <c r="C110" s="171" t="n"/>
+      <c r="D110" s="172" t="n"/>
+      <c r="E110" s="161" t="n"/>
+      <c r="F110" s="158" t="n"/>
     </row>
     <row r="111" ht="15" customHeight="1">
       <c r="B111" s="24" t="n"/>
-      <c r="C111" s="173" t="n"/>
-      <c r="D111" s="174" t="n"/>
-      <c r="E111" s="162" t="n"/>
-      <c r="F111" s="163" t="n"/>
+      <c r="C111" s="171" t="n"/>
+      <c r="D111" s="172" t="n"/>
+      <c r="E111" s="161" t="n"/>
+      <c r="F111" s="158" t="n"/>
     </row>
     <row r="112" ht="15" customHeight="1">
       <c r="B112" s="24" t="n"/>
-      <c r="C112" s="173" t="n"/>
-      <c r="D112" s="174" t="n"/>
-      <c r="E112" s="162" t="n"/>
-      <c r="F112" s="163" t="n"/>
+      <c r="C112" s="171" t="n"/>
+      <c r="D112" s="172" t="n"/>
+      <c r="E112" s="161" t="n"/>
+      <c r="F112" s="158" t="n"/>
     </row>
     <row r="113" ht="15" customHeight="1">
       <c r="B113" s="24" t="n"/>
-      <c r="C113" s="173" t="n"/>
-      <c r="D113" s="174" t="n"/>
-      <c r="E113" s="162" t="n"/>
-      <c r="F113" s="163" t="n"/>
+      <c r="C113" s="171" t="n"/>
+      <c r="D113" s="172" t="n"/>
+      <c r="E113" s="161" t="n"/>
+      <c r="F113" s="158" t="n"/>
     </row>
     <row r="114" ht="15" customHeight="1">
       <c r="B114" s="24" t="n"/>
-      <c r="C114" s="173" t="n"/>
-      <c r="D114" s="174" t="n"/>
-      <c r="E114" s="162" t="n"/>
-      <c r="F114" s="163" t="n"/>
+      <c r="C114" s="171" t="n"/>
+      <c r="D114" s="172" t="n"/>
+      <c r="E114" s="161" t="n"/>
+      <c r="F114" s="158" t="n"/>
     </row>
     <row r="115" ht="15" customHeight="1">
       <c r="B115" s="24" t="n"/>
-      <c r="C115" s="173" t="n"/>
-      <c r="D115" s="174" t="n"/>
-      <c r="E115" s="162" t="n"/>
-      <c r="F115" s="163" t="n"/>
+      <c r="C115" s="171" t="n"/>
+      <c r="D115" s="172" t="n"/>
+      <c r="E115" s="161" t="n"/>
+      <c r="F115" s="158" t="n"/>
     </row>
     <row r="116" ht="15" customHeight="1">
       <c r="B116" s="24" t="n"/>
-      <c r="C116" s="173" t="n"/>
-      <c r="D116" s="174" t="n"/>
-      <c r="E116" s="162" t="n"/>
-      <c r="F116" s="163" t="n"/>
+      <c r="C116" s="171" t="n"/>
+      <c r="D116" s="172" t="n"/>
+      <c r="E116" s="161" t="n"/>
+      <c r="F116" s="158" t="n"/>
     </row>
     <row r="117" ht="15" customHeight="1">
       <c r="B117" s="24" t="n"/>
-      <c r="C117" s="173" t="n"/>
-      <c r="D117" s="174" t="n"/>
-      <c r="E117" s="162" t="n"/>
-      <c r="F117" s="163" t="n"/>
+      <c r="C117" s="171" t="n"/>
+      <c r="D117" s="172" t="n"/>
+      <c r="E117" s="161" t="n"/>
+      <c r="F117" s="158" t="n"/>
     </row>
     <row r="118" ht="15" customHeight="1">
       <c r="B118" s="24" t="n"/>
-      <c r="C118" s="173" t="n"/>
-      <c r="D118" s="174" t="n"/>
-      <c r="E118" s="162" t="n"/>
-      <c r="F118" s="163" t="n"/>
+      <c r="C118" s="171" t="n"/>
+      <c r="D118" s="172" t="n"/>
+      <c r="E118" s="161" t="n"/>
+      <c r="F118" s="158" t="n"/>
     </row>
     <row r="119" ht="15" customHeight="1">
       <c r="B119" s="24" t="n"/>
-      <c r="C119" s="173" t="n"/>
-      <c r="D119" s="174" t="n"/>
-      <c r="E119" s="162" t="n"/>
-      <c r="F119" s="163" t="n"/>
+      <c r="C119" s="171" t="n"/>
+      <c r="D119" s="172" t="n"/>
+      <c r="E119" s="161" t="n"/>
+      <c r="F119" s="158" t="n"/>
     </row>
     <row r="120" ht="15" customHeight="1">
       <c r="B120" s="24" t="n"/>
-      <c r="C120" s="173" t="n"/>
-      <c r="D120" s="174" t="n"/>
-      <c r="E120" s="162" t="n"/>
-      <c r="F120" s="163" t="n"/>
+      <c r="C120" s="171" t="n"/>
+      <c r="D120" s="172" t="n"/>
+      <c r="E120" s="161" t="n"/>
+      <c r="F120" s="158" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1">
       <c r="B121" s="24" t="n"/>
-      <c r="C121" s="173" t="n"/>
-      <c r="D121" s="174" t="n"/>
+      <c r="C121" s="171" t="n"/>
+      <c r="D121" s="172" t="n"/>
       <c r="E121" s="32" t="n"/>
-      <c r="F121" s="163" t="n"/>
+      <c r="F121" s="158" t="n"/>
     </row>
     <row r="122" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B122" s="74" t="inlineStr">
@@ -2982,7 +2964,7 @@
       <c r="C122" s="27" t="n"/>
       <c r="D122" s="27" t="n"/>
       <c r="E122" s="27" t="n"/>
-      <c r="F122" s="168">
+      <c r="F122" s="166">
         <f>SUM(F108:F121)</f>
         <v/>
       </c>
@@ -2990,7 +2972,7 @@
       <c r="Q122" s="28" t="n"/>
     </row>
     <row r="123" ht="15" customFormat="1" customHeight="1" s="10">
-      <c r="F123" s="175" t="n"/>
+      <c r="F123" s="173" t="n"/>
       <c r="H123" s="70" t="n"/>
       <c r="Q123" s="28" t="n"/>
     </row>
@@ -3030,154 +3012,154 @@
     </row>
     <row r="126" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B126" s="24" t="n"/>
-      <c r="C126" s="173" t="n"/>
-      <c r="D126" s="174" t="n"/>
-      <c r="E126" s="162" t="n"/>
-      <c r="F126" s="163" t="n"/>
+      <c r="C126" s="171" t="n"/>
+      <c r="D126" s="172" t="n"/>
+      <c r="E126" s="161" t="n"/>
+      <c r="F126" s="158" t="n"/>
       <c r="H126" s="66" t="n"/>
       <c r="Q126" s="28" t="n"/>
     </row>
     <row r="127" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B127" s="24" t="n"/>
-      <c r="C127" s="173" t="n"/>
-      <c r="D127" s="174" t="n"/>
-      <c r="E127" s="162" t="n"/>
-      <c r="F127" s="163" t="n"/>
+      <c r="C127" s="171" t="n"/>
+      <c r="D127" s="172" t="n"/>
+      <c r="E127" s="161" t="n"/>
+      <c r="F127" s="158" t="n"/>
       <c r="H127" s="66" t="n"/>
       <c r="Q127" s="28" t="n"/>
     </row>
     <row r="128" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B128" s="24" t="n"/>
-      <c r="C128" s="173" t="n"/>
-      <c r="D128" s="174" t="n"/>
-      <c r="E128" s="162" t="n"/>
-      <c r="F128" s="163" t="n"/>
+      <c r="C128" s="171" t="n"/>
+      <c r="D128" s="172" t="n"/>
+      <c r="E128" s="161" t="n"/>
+      <c r="F128" s="158" t="n"/>
       <c r="H128" s="66" t="n"/>
       <c r="Q128" s="28" t="n"/>
     </row>
     <row r="129" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B129" s="24" t="n"/>
-      <c r="C129" s="173" t="n"/>
-      <c r="D129" s="174" t="n"/>
-      <c r="E129" s="162" t="n"/>
-      <c r="F129" s="163" t="n"/>
+      <c r="C129" s="171" t="n"/>
+      <c r="D129" s="172" t="n"/>
+      <c r="E129" s="161" t="n"/>
+      <c r="F129" s="158" t="n"/>
       <c r="H129" s="66" t="n"/>
       <c r="Q129" s="28" t="n"/>
     </row>
     <row r="130" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B130" s="24" t="n"/>
-      <c r="C130" s="173" t="n"/>
-      <c r="D130" s="174" t="n"/>
-      <c r="E130" s="162" t="n"/>
-      <c r="F130" s="163" t="n"/>
+      <c r="C130" s="171" t="n"/>
+      <c r="D130" s="172" t="n"/>
+      <c r="E130" s="161" t="n"/>
+      <c r="F130" s="158" t="n"/>
       <c r="H130" s="66" t="n"/>
       <c r="Q130" s="28" t="n"/>
     </row>
     <row r="131" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B131" s="24" t="n"/>
-      <c r="C131" s="173" t="n"/>
-      <c r="D131" s="174" t="n"/>
-      <c r="E131" s="162" t="n"/>
-      <c r="F131" s="163" t="n"/>
+      <c r="C131" s="171" t="n"/>
+      <c r="D131" s="172" t="n"/>
+      <c r="E131" s="161" t="n"/>
+      <c r="F131" s="158" t="n"/>
       <c r="H131" s="66" t="n"/>
       <c r="Q131" s="28" t="n"/>
     </row>
     <row r="132" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B132" s="24" t="n"/>
-      <c r="C132" s="173" t="n"/>
-      <c r="D132" s="174" t="n"/>
-      <c r="E132" s="162" t="n"/>
-      <c r="F132" s="163" t="n"/>
+      <c r="C132" s="171" t="n"/>
+      <c r="D132" s="172" t="n"/>
+      <c r="E132" s="161" t="n"/>
+      <c r="F132" s="158" t="n"/>
       <c r="H132" s="66" t="n"/>
       <c r="Q132" s="28" t="n"/>
     </row>
     <row r="133" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B133" s="24" t="n"/>
-      <c r="C133" s="173" t="n"/>
-      <c r="D133" s="174" t="n"/>
-      <c r="E133" s="162" t="n"/>
-      <c r="F133" s="163" t="n"/>
+      <c r="C133" s="171" t="n"/>
+      <c r="D133" s="172" t="n"/>
+      <c r="E133" s="161" t="n"/>
+      <c r="F133" s="158" t="n"/>
       <c r="H133" s="66" t="n"/>
       <c r="Q133" s="28" t="n"/>
     </row>
     <row r="134" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B134" s="24" t="n"/>
-      <c r="C134" s="173" t="n"/>
-      <c r="D134" s="174" t="n"/>
-      <c r="E134" s="162" t="n"/>
-      <c r="F134" s="163" t="n"/>
+      <c r="C134" s="171" t="n"/>
+      <c r="D134" s="172" t="n"/>
+      <c r="E134" s="161" t="n"/>
+      <c r="F134" s="158" t="n"/>
       <c r="H134" s="66" t="n"/>
       <c r="Q134" s="28" t="n"/>
     </row>
     <row r="135" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B135" s="24" t="n"/>
-      <c r="C135" s="173" t="n"/>
-      <c r="D135" s="174" t="n"/>
-      <c r="E135" s="162" t="n"/>
-      <c r="F135" s="163" t="n"/>
+      <c r="C135" s="171" t="n"/>
+      <c r="D135" s="172" t="n"/>
+      <c r="E135" s="161" t="n"/>
+      <c r="F135" s="158" t="n"/>
       <c r="H135" s="66" t="n"/>
       <c r="Q135" s="28" t="n"/>
     </row>
     <row r="136" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B136" s="24" t="n"/>
-      <c r="C136" s="173" t="n"/>
-      <c r="D136" s="174" t="n"/>
-      <c r="E136" s="162" t="n"/>
-      <c r="F136" s="163" t="n"/>
+      <c r="C136" s="171" t="n"/>
+      <c r="D136" s="172" t="n"/>
+      <c r="E136" s="161" t="n"/>
+      <c r="F136" s="158" t="n"/>
       <c r="H136" s="66" t="n"/>
       <c r="Q136" s="28" t="n"/>
     </row>
     <row r="137" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B137" s="24" t="n"/>
-      <c r="C137" s="173" t="n"/>
-      <c r="D137" s="174" t="n"/>
-      <c r="E137" s="162" t="n"/>
-      <c r="F137" s="163" t="n"/>
+      <c r="C137" s="171" t="n"/>
+      <c r="D137" s="172" t="n"/>
+      <c r="E137" s="161" t="n"/>
+      <c r="F137" s="158" t="n"/>
       <c r="H137" s="66" t="n"/>
       <c r="Q137" s="28" t="n"/>
     </row>
     <row r="138" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B138" s="24" t="n"/>
-      <c r="C138" s="173" t="n"/>
-      <c r="D138" s="174" t="n"/>
-      <c r="E138" s="162" t="n"/>
-      <c r="F138" s="163" t="n"/>
+      <c r="C138" s="171" t="n"/>
+      <c r="D138" s="172" t="n"/>
+      <c r="E138" s="161" t="n"/>
+      <c r="F138" s="158" t="n"/>
       <c r="H138" s="70" t="n"/>
       <c r="Q138" s="28" t="n"/>
     </row>
     <row r="139" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B139" s="24" t="n"/>
-      <c r="C139" s="173" t="n"/>
-      <c r="D139" s="174" t="n"/>
-      <c r="E139" s="162" t="n"/>
-      <c r="F139" s="163" t="n"/>
+      <c r="C139" s="171" t="n"/>
+      <c r="D139" s="172" t="n"/>
+      <c r="E139" s="161" t="n"/>
+      <c r="F139" s="158" t="n"/>
       <c r="H139" s="70" t="n"/>
       <c r="Q139" s="28" t="n"/>
     </row>
     <row r="140" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B140" s="24" t="n"/>
-      <c r="C140" s="173" t="n"/>
-      <c r="D140" s="174" t="n"/>
-      <c r="E140" s="162" t="n"/>
-      <c r="F140" s="163" t="n"/>
+      <c r="C140" s="171" t="n"/>
+      <c r="D140" s="172" t="n"/>
+      <c r="E140" s="161" t="n"/>
+      <c r="F140" s="158" t="n"/>
       <c r="H140" s="70" t="n"/>
       <c r="Q140" s="28" t="n"/>
     </row>
     <row r="141" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B141" s="24" t="n"/>
-      <c r="C141" s="173" t="n"/>
-      <c r="D141" s="174" t="n"/>
-      <c r="E141" s="162" t="n"/>
-      <c r="F141" s="163" t="n"/>
+      <c r="C141" s="171" t="n"/>
+      <c r="D141" s="172" t="n"/>
+      <c r="E141" s="161" t="n"/>
+      <c r="F141" s="158" t="n"/>
       <c r="H141" s="70" t="n"/>
       <c r="Q141" s="28" t="n"/>
     </row>
     <row r="142" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B142" s="24" t="n"/>
-      <c r="C142" s="173" t="n"/>
-      <c r="D142" s="174" t="n"/>
+      <c r="C142" s="171" t="n"/>
+      <c r="D142" s="172" t="n"/>
       <c r="E142" s="32" t="n"/>
-      <c r="F142" s="163" t="n"/>
+      <c r="F142" s="158" t="n"/>
       <c r="H142" s="70" t="n"/>
       <c r="Q142" s="28" t="n"/>
     </row>
@@ -3190,7 +3172,7 @@
       <c r="C143" s="27" t="n"/>
       <c r="D143" s="27" t="n"/>
       <c r="E143" s="27" t="n"/>
-      <c r="F143" s="168">
+      <c r="F143" s="166">
         <f>SUM(F126:F142)</f>
         <v/>
       </c>
@@ -3229,122 +3211,122 @@
     </row>
     <row r="147" ht="15" customHeight="1">
       <c r="B147" s="24" t="n"/>
-      <c r="C147" s="173" t="n"/>
-      <c r="D147" s="174" t="n"/>
-      <c r="E147" s="162" t="n"/>
-      <c r="F147" s="163" t="n"/>
+      <c r="C147" s="171" t="n"/>
+      <c r="D147" s="172" t="n"/>
+      <c r="E147" s="161" t="n"/>
+      <c r="F147" s="158" t="n"/>
     </row>
     <row r="148" ht="15" customHeight="1">
       <c r="B148" s="33" t="n"/>
-      <c r="C148" s="176" t="n"/>
-      <c r="D148" s="177" t="n"/>
+      <c r="C148" s="174" t="n"/>
+      <c r="D148" s="175" t="n"/>
       <c r="E148" s="36" t="n"/>
-      <c r="F148" s="163" t="n"/>
+      <c r="F148" s="158" t="n"/>
     </row>
     <row r="149" ht="15" customHeight="1">
       <c r="B149" s="33" t="n"/>
-      <c r="C149" s="173" t="n"/>
-      <c r="D149" s="174" t="n"/>
+      <c r="C149" s="171" t="n"/>
+      <c r="D149" s="172" t="n"/>
       <c r="E149" s="36" t="n"/>
-      <c r="F149" s="163" t="n"/>
+      <c r="F149" s="158" t="n"/>
     </row>
     <row r="150" ht="15" customHeight="1">
       <c r="B150" s="33" t="n"/>
-      <c r="C150" s="173" t="n"/>
-      <c r="D150" s="174" t="n"/>
+      <c r="C150" s="171" t="n"/>
+      <c r="D150" s="172" t="n"/>
       <c r="E150" s="36" t="n"/>
-      <c r="F150" s="163" t="n"/>
+      <c r="F150" s="158" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1">
       <c r="B151" s="33" t="n"/>
-      <c r="C151" s="173" t="n"/>
-      <c r="D151" s="174" t="n"/>
+      <c r="C151" s="171" t="n"/>
+      <c r="D151" s="172" t="n"/>
       <c r="E151" s="36" t="n"/>
-      <c r="F151" s="163" t="n"/>
+      <c r="F151" s="158" t="n"/>
     </row>
     <row r="152" ht="15" customHeight="1">
       <c r="B152" s="33" t="n"/>
-      <c r="C152" s="173" t="n"/>
-      <c r="D152" s="174" t="n"/>
+      <c r="C152" s="171" t="n"/>
+      <c r="D152" s="172" t="n"/>
       <c r="E152" s="36" t="n"/>
-      <c r="F152" s="163" t="n"/>
+      <c r="F152" s="158" t="n"/>
     </row>
     <row r="153" ht="15" customHeight="1">
       <c r="B153" s="33" t="n"/>
-      <c r="C153" s="173" t="n"/>
-      <c r="D153" s="174" t="n"/>
+      <c r="C153" s="171" t="n"/>
+      <c r="D153" s="172" t="n"/>
       <c r="E153" s="36" t="n"/>
-      <c r="F153" s="163" t="n"/>
+      <c r="F153" s="158" t="n"/>
     </row>
     <row r="154" ht="15" customHeight="1">
       <c r="B154" s="33" t="n"/>
-      <c r="C154" s="173" t="n"/>
-      <c r="D154" s="174" t="n"/>
+      <c r="C154" s="171" t="n"/>
+      <c r="D154" s="172" t="n"/>
       <c r="E154" s="36" t="n"/>
-      <c r="F154" s="163" t="n"/>
+      <c r="F154" s="158" t="n"/>
     </row>
     <row r="155" ht="15" customHeight="1">
       <c r="B155" s="33" t="n"/>
-      <c r="C155" s="173" t="n"/>
-      <c r="D155" s="174" t="n"/>
+      <c r="C155" s="171" t="n"/>
+      <c r="D155" s="172" t="n"/>
       <c r="E155" s="36" t="n"/>
-      <c r="F155" s="163" t="n"/>
+      <c r="F155" s="158" t="n"/>
     </row>
     <row r="156" ht="15" customHeight="1">
       <c r="B156" s="33" t="n"/>
-      <c r="C156" s="173" t="n"/>
-      <c r="D156" s="174" t="n"/>
+      <c r="C156" s="171" t="n"/>
+      <c r="D156" s="172" t="n"/>
       <c r="E156" s="36" t="n"/>
-      <c r="F156" s="163" t="n"/>
+      <c r="F156" s="158" t="n"/>
     </row>
     <row r="157" ht="15" customHeight="1">
       <c r="B157" s="33" t="n"/>
-      <c r="C157" s="173" t="n"/>
-      <c r="D157" s="174" t="n"/>
+      <c r="C157" s="171" t="n"/>
+      <c r="D157" s="172" t="n"/>
       <c r="E157" s="36" t="n"/>
-      <c r="F157" s="163" t="n"/>
+      <c r="F157" s="158" t="n"/>
     </row>
     <row r="158" ht="15" customHeight="1">
       <c r="B158" s="33" t="n"/>
-      <c r="C158" s="173" t="n"/>
-      <c r="D158" s="174" t="n"/>
+      <c r="C158" s="171" t="n"/>
+      <c r="D158" s="172" t="n"/>
       <c r="E158" s="36" t="n"/>
-      <c r="F158" s="163" t="n"/>
+      <c r="F158" s="158" t="n"/>
     </row>
     <row r="159" ht="15" customHeight="1">
       <c r="B159" s="33" t="n"/>
-      <c r="C159" s="173" t="n"/>
-      <c r="D159" s="174" t="n"/>
+      <c r="C159" s="171" t="n"/>
+      <c r="D159" s="172" t="n"/>
       <c r="E159" s="36" t="n"/>
-      <c r="F159" s="163" t="n"/>
+      <c r="F159" s="158" t="n"/>
     </row>
     <row r="160" ht="15" customHeight="1">
       <c r="B160" s="33" t="n"/>
-      <c r="C160" s="173" t="n"/>
-      <c r="D160" s="174" t="n"/>
+      <c r="C160" s="171" t="n"/>
+      <c r="D160" s="172" t="n"/>
       <c r="E160" s="36" t="n"/>
-      <c r="F160" s="163" t="n"/>
+      <c r="F160" s="158" t="n"/>
     </row>
     <row r="161" ht="15" customHeight="1">
       <c r="B161" s="33" t="n"/>
-      <c r="C161" s="173" t="n"/>
-      <c r="D161" s="174" t="n"/>
+      <c r="C161" s="171" t="n"/>
+      <c r="D161" s="172" t="n"/>
       <c r="E161" s="36" t="n"/>
-      <c r="F161" s="163" t="n"/>
+      <c r="F161" s="158" t="n"/>
     </row>
     <row r="162" ht="15" customHeight="1">
       <c r="B162" s="24" t="n"/>
-      <c r="C162" s="173" t="n"/>
-      <c r="D162" s="174" t="n"/>
+      <c r="C162" s="171" t="n"/>
+      <c r="D162" s="172" t="n"/>
       <c r="E162" s="32" t="n"/>
-      <c r="F162" s="163" t="n"/>
+      <c r="F162" s="158" t="n"/>
     </row>
     <row r="163" ht="15" customHeight="1">
       <c r="B163" s="24" t="n"/>
-      <c r="C163" s="173" t="n"/>
-      <c r="D163" s="174" t="n"/>
+      <c r="C163" s="171" t="n"/>
+      <c r="D163" s="172" t="n"/>
       <c r="E163" s="32" t="n"/>
-      <c r="F163" s="178" t="n"/>
+      <c r="F163" s="176" t="n"/>
     </row>
     <row r="164" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="B164" s="27" t="inlineStr">
@@ -3355,7 +3337,7 @@
       <c r="C164" s="27" t="n"/>
       <c r="D164" s="27" t="n"/>
       <c r="E164" s="27" t="n"/>
-      <c r="F164" s="168">
+      <c r="F164" s="166">
         <f>SUM(F147:F163)</f>
         <v/>
       </c>
@@ -3394,159 +3376,159 @@
     </row>
     <row r="168" ht="15" customHeight="1">
       <c r="B168" s="33" t="n"/>
-      <c r="C168" s="176" t="n"/>
-      <c r="D168" s="177" t="n"/>
-      <c r="E168" s="162" t="n"/>
-      <c r="F168" s="179" t="n"/>
+      <c r="C168" s="174" t="n"/>
+      <c r="D168" s="175" t="n"/>
+      <c r="E168" s="161" t="n"/>
+      <c r="F168" s="177" t="n"/>
     </row>
     <row r="169" ht="15" customHeight="1">
       <c r="B169" s="33" t="n"/>
-      <c r="C169" s="176" t="n"/>
-      <c r="D169" s="177" t="n"/>
+      <c r="C169" s="174" t="n"/>
+      <c r="D169" s="175" t="n"/>
       <c r="E169" s="36" t="n"/>
-      <c r="F169" s="180" t="n"/>
+      <c r="F169" s="178" t="n"/>
     </row>
     <row r="170" ht="15" customHeight="1">
       <c r="B170" s="24" t="n"/>
-      <c r="C170" s="176" t="n"/>
-      <c r="D170" s="177" t="n"/>
+      <c r="C170" s="174" t="n"/>
+      <c r="D170" s="175" t="n"/>
       <c r="E170" s="36" t="n"/>
-      <c r="F170" s="180" t="n"/>
+      <c r="F170" s="178" t="n"/>
       <c r="H170" s="4" t="n"/>
       <c r="Q170" s="4" t="n"/>
     </row>
     <row r="171" ht="15" customHeight="1">
       <c r="B171" s="24" t="n"/>
-      <c r="C171" s="176" t="n"/>
-      <c r="D171" s="177" t="n"/>
+      <c r="C171" s="174" t="n"/>
+      <c r="D171" s="175" t="n"/>
       <c r="E171" s="36" t="n"/>
-      <c r="F171" s="180" t="n"/>
+      <c r="F171" s="178" t="n"/>
       <c r="H171" s="4" t="n"/>
       <c r="Q171" s="4" t="n"/>
     </row>
     <row r="172" ht="15" customHeight="1">
       <c r="B172" s="33" t="n"/>
-      <c r="C172" s="176" t="n"/>
-      <c r="D172" s="177" t="n"/>
+      <c r="C172" s="174" t="n"/>
+      <c r="D172" s="175" t="n"/>
       <c r="E172" s="36" t="n"/>
-      <c r="F172" s="180" t="n"/>
+      <c r="F172" s="178" t="n"/>
       <c r="H172" s="4" t="n"/>
       <c r="Q172" s="4" t="n"/>
     </row>
     <row r="173" ht="15" customHeight="1">
       <c r="B173" s="33" t="n"/>
-      <c r="C173" s="176" t="n"/>
-      <c r="D173" s="177" t="n"/>
+      <c r="C173" s="174" t="n"/>
+      <c r="D173" s="175" t="n"/>
       <c r="E173" s="36" t="n"/>
-      <c r="F173" s="180" t="n"/>
+      <c r="F173" s="178" t="n"/>
       <c r="H173" s="4" t="n"/>
       <c r="Q173" s="4" t="n"/>
     </row>
     <row r="174" ht="15" customHeight="1">
       <c r="B174" s="33" t="n"/>
-      <c r="C174" s="176" t="n"/>
-      <c r="D174" s="177" t="n"/>
+      <c r="C174" s="174" t="n"/>
+      <c r="D174" s="175" t="n"/>
       <c r="E174" s="36" t="n"/>
-      <c r="F174" s="180" t="n"/>
+      <c r="F174" s="178" t="n"/>
       <c r="H174" s="4" t="n"/>
       <c r="Q174" s="4" t="n"/>
     </row>
     <row r="175" ht="15" customHeight="1">
       <c r="B175" s="33" t="n"/>
-      <c r="C175" s="176" t="n"/>
-      <c r="D175" s="177" t="n"/>
+      <c r="C175" s="174" t="n"/>
+      <c r="D175" s="175" t="n"/>
       <c r="E175" s="36" t="n"/>
-      <c r="F175" s="180" t="n"/>
+      <c r="F175" s="178" t="n"/>
       <c r="H175" s="4" t="n"/>
       <c r="Q175" s="4" t="n"/>
     </row>
     <row r="176" ht="15" customHeight="1">
       <c r="B176" s="33" t="n"/>
-      <c r="C176" s="176" t="n"/>
-      <c r="D176" s="177" t="n"/>
+      <c r="C176" s="174" t="n"/>
+      <c r="D176" s="175" t="n"/>
       <c r="E176" s="36" t="n"/>
-      <c r="F176" s="180" t="n"/>
+      <c r="F176" s="178" t="n"/>
       <c r="H176" s="4" t="n"/>
       <c r="Q176" s="4" t="n"/>
     </row>
     <row r="177" ht="15" customHeight="1">
       <c r="B177" s="33" t="n"/>
-      <c r="C177" s="176" t="n"/>
-      <c r="D177" s="177" t="n"/>
+      <c r="C177" s="174" t="n"/>
+      <c r="D177" s="175" t="n"/>
       <c r="E177" s="36" t="n"/>
-      <c r="F177" s="180" t="n"/>
+      <c r="F177" s="178" t="n"/>
       <c r="H177" s="4" t="n"/>
       <c r="Q177" s="4" t="n"/>
     </row>
     <row r="178" ht="15" customHeight="1">
       <c r="B178" s="33" t="n"/>
-      <c r="C178" s="176" t="n"/>
-      <c r="D178" s="177" t="n"/>
+      <c r="C178" s="174" t="n"/>
+      <c r="D178" s="175" t="n"/>
       <c r="E178" s="36" t="n"/>
-      <c r="F178" s="180" t="n"/>
+      <c r="F178" s="178" t="n"/>
       <c r="H178" s="4" t="n"/>
       <c r="Q178" s="4" t="n"/>
     </row>
     <row r="179" ht="15" customHeight="1">
       <c r="B179" s="33" t="n"/>
-      <c r="C179" s="176" t="n"/>
-      <c r="D179" s="177" t="n"/>
+      <c r="C179" s="174" t="n"/>
+      <c r="D179" s="175" t="n"/>
       <c r="E179" s="36" t="n"/>
-      <c r="F179" s="180" t="n"/>
+      <c r="F179" s="178" t="n"/>
       <c r="H179" s="4" t="n"/>
       <c r="Q179" s="4" t="n"/>
     </row>
     <row r="180" ht="15" customHeight="1">
       <c r="B180" s="33" t="n"/>
-      <c r="C180" s="176" t="n"/>
-      <c r="D180" s="177" t="n"/>
+      <c r="C180" s="174" t="n"/>
+      <c r="D180" s="175" t="n"/>
       <c r="E180" s="36" t="n"/>
-      <c r="F180" s="180" t="n"/>
+      <c r="F180" s="178" t="n"/>
       <c r="H180" s="4" t="n"/>
       <c r="Q180" s="4" t="n"/>
     </row>
     <row r="181" ht="15" customHeight="1">
       <c r="B181" s="33" t="n"/>
-      <c r="C181" s="176" t="n"/>
-      <c r="D181" s="177" t="n"/>
+      <c r="C181" s="174" t="n"/>
+      <c r="D181" s="175" t="n"/>
       <c r="E181" s="36" t="n"/>
-      <c r="F181" s="180" t="n"/>
+      <c r="F181" s="178" t="n"/>
       <c r="H181" s="4" t="n"/>
       <c r="Q181" s="4" t="n"/>
     </row>
     <row r="182" ht="15" customHeight="1">
       <c r="B182" s="33" t="n"/>
-      <c r="C182" s="176" t="n"/>
-      <c r="D182" s="177" t="n"/>
+      <c r="C182" s="174" t="n"/>
+      <c r="D182" s="175" t="n"/>
       <c r="E182" s="36" t="n"/>
-      <c r="F182" s="180" t="n"/>
+      <c r="F182" s="178" t="n"/>
       <c r="H182" s="4" t="n"/>
       <c r="Q182" s="4" t="n"/>
     </row>
     <row r="183" ht="15" customHeight="1">
       <c r="B183" s="33" t="n"/>
-      <c r="C183" s="176" t="n"/>
-      <c r="D183" s="177" t="n"/>
+      <c r="C183" s="174" t="n"/>
+      <c r="D183" s="175" t="n"/>
       <c r="E183" s="36" t="n"/>
-      <c r="F183" s="180" t="n"/>
+      <c r="F183" s="178" t="n"/>
       <c r="H183" s="4" t="n"/>
       <c r="Q183" s="4" t="n"/>
     </row>
     <row r="184" ht="15" customHeight="1">
       <c r="B184" s="33" t="n"/>
-      <c r="C184" s="176" t="n"/>
-      <c r="D184" s="177" t="n"/>
+      <c r="C184" s="174" t="n"/>
+      <c r="D184" s="175" t="n"/>
       <c r="E184" s="36" t="n"/>
-      <c r="F184" s="180" t="n"/>
+      <c r="F184" s="178" t="n"/>
       <c r="H184" s="4" t="n"/>
       <c r="Q184" s="4" t="n"/>
     </row>
     <row r="185" ht="15" customHeight="1">
       <c r="B185" s="33" t="n"/>
-      <c r="C185" s="176" t="n"/>
-      <c r="D185" s="177" t="n"/>
+      <c r="C185" s="174" t="n"/>
+      <c r="D185" s="175" t="n"/>
       <c r="E185" s="36" t="n"/>
-      <c r="F185" s="180" t="n"/>
+      <c r="F185" s="178" t="n"/>
       <c r="H185" s="4" t="n"/>
       <c r="Q185" s="4" t="n"/>
     </row>
@@ -3559,7 +3541,7 @@
       <c r="C186" s="38" t="n"/>
       <c r="D186" s="38" t="n"/>
       <c r="E186" s="38" t="n"/>
-      <c r="F186" s="181">
+      <c r="F186" s="179">
         <f>SUM(F168:F185)</f>
         <v/>
       </c>
@@ -3576,7 +3558,7 @@
       <c r="C187" s="39" t="n"/>
       <c r="D187" s="39" t="n"/>
       <c r="E187" s="39" t="n"/>
-      <c r="F187" s="182" t="n"/>
+      <c r="F187" s="180" t="n"/>
       <c r="G187" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -3590,7 +3572,7 @@
       <c r="C188" s="1" t="n"/>
       <c r="D188" s="1" t="n"/>
       <c r="E188" s="1" t="n"/>
-      <c r="F188" s="183" t="n"/>
+      <c r="F188" s="181" t="n"/>
       <c r="H188" s="4" t="n"/>
       <c r="Q188" s="4" t="n"/>
     </row>
@@ -3599,13 +3581,13 @@
       <c r="C189" s="1" t="n"/>
       <c r="D189" s="1" t="n"/>
       <c r="E189" s="1" t="n"/>
-      <c r="F189" s="184" t="n"/>
+      <c r="F189" s="182" t="n"/>
       <c r="H189" s="4" t="n"/>
       <c r="Q189" s="4" t="n"/>
     </row>
     <row r="190" ht="15" customHeight="1">
       <c r="B190" s="42" t="n"/>
-      <c r="F190" s="185" t="n"/>
+      <c r="F190" s="183" t="n"/>
       <c r="H190" s="4" t="n"/>
       <c r="Q190" s="4" t="n"/>
     </row>

</xml_diff>